<commit_message>
Added Excel for new rock type mapping
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Yukon_Geothermal_Springs.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/Yukon_Geothermal_Springs.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\Gesammelte_Datenbanken\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94a36cc37384f3e2/SPEICHER/Hochschule/7. Semester/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B63BADE5-BEDD-4E66-85D0-1B7C04C396AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>

</xml_diff>